<commit_message>
Statements: kinds of lines, and loan installments split into principal and interest
- The Ziraat Bankası template tells card purchases, transfers, the bank's
  fees, cash withdrawals, bill payments and loan installments apart, and
  reads the payee of each (the company of a bill, the bank for its fees).
- An installment line of a loan defined with its number is booked as that
  loan's payment, split into principal, interest and taxes. Unknown loan
  numbers are reported; lines dated before the loan's start in the ledger are
  refused.
- The made-up statements have one line of each kind.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/ziraat_statement.xlsx
+++ b/tests/fixtures/ziraat_statement.xlsx
@@ -113,7 +113,7 @@
         <x:v>-1750</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>41724.55</x:v>
+        <x:v>35086.32</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -130,7 +130,7 @@
         <x:v>5000</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>43474.55</x:v>
+        <x:v>36836.32</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -147,7 +147,24 @@
         <x:v>-2000.00</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>38474.55</x:v>
+        <x:v>31836.32</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="0" t="str">
+        <x:v>18.09.2026</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>F18550</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>ÖRNEK KİŞİ KİRA PAYI FAST</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>33836.32</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -164,7 +181,7 @@
         <x:v>-85.50</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>40474.55</x:v>
+        <x:v>30836.32</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -181,7 +198,7 @@
         <x:v>-85.50</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>40560.05</x:v>
+        <x:v>30921.82</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -198,7 +215,41 @@
         <x:v>-229.99</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>40645.55</x:v>
+        <x:v>31007.32</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="0" t="str">
+        <x:v>13.09.2026</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>F13440</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>12345678-0001 hesap 5. taksit ödeme tutarı</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>-6924.20</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>31237.31</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="0" t="str">
+        <x:v>11.09.2026</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>F11330</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>ÖRNEK ELEKTRİK PERAKENDE/ Abone no: 10000001 / Fatura no: 2000002 / Fatura Tutarı: 456,78 / Son Ödeme: 18.09.2026</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>-456.78</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>38161.51</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -215,7 +266,24 @@
         <x:v>-389.9</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>40875.54</x:v>
+        <x:v>38618.29</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="0" t="str">
+        <x:v>07.09.2026</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>F07250</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>ATM PARA ÇEKME KART:4000****0000 ATM: Z0042 ÖRNEK ŞUBESİ</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>-2250</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>39008.19</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -232,7 +300,7 @@
         <x:v>-15000</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>41265.44</x:v>
+        <x:v>41258.19</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -249,7 +317,41 @@
         <x:v>-1234.56</x:v>
       </x:c>
       <x:c s="2" t="n">
-        <x:v>56265.44</x:v>
+        <x:v>56258.19</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="0" t="str">
+        <x:v>02.09.2026</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>F02151</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>BSMV TUTARI</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>-0.35</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>57492.75</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="0" t="str">
+        <x:v>02.09.2026</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>F02150</x:v>
+      </x:c>
+      <x:c s="0" t="str">
+        <x:v>MESAJ ÜCRETİ TUTARI</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>-6.90</x:v>
+      </x:c>
+      <x:c s="2" t="n">
+        <x:v>57493.10</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -281,10 +383,10 @@
       <x:c s="0"/>
       <x:c s="0"/>
       <x:c s="1" t="str">
-        <x:v>Borç:-20.775,45</x:v>
-      </x:c>
-      <x:c s="1" t="str">
-        <x:v>Alacak:50.000</x:v>
+        <x:v>Borç:-30.413,68</x:v>
+      </x:c>
+      <x:c s="1" t="str">
+        <x:v>Alacak:53.000</x:v>
       </x:c>
     </x:row>
     <x:row/>

</xml_diff>